<commit_message>
fixing cable units bug from rotorD to km (#207)
* fixing cable units bug from rotorD to km

* remove extra indent

* update changelog

---------

Co-authored-by: Garrett Barter <garrett.barter@nrel.gov>
Co-authored-by: RHammond2 <13874373+RHammond2@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/project_input_template/project_data/ge15_expected_validation.xlsx
+++ b/project_input_template/project_data/ge15_expected_validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pcrook\nrel\github\LandBOSSE\input\project_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gbarter/devel/LandBOSSE/project_input_template/project_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B79682-D817-49EC-8218-147192497AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EB1AE9-BDEA-434B-8557-872E6F73BA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17520" yWindow="3320" windowWidth="34080" windowHeight="18820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="costs_by_module_type_operation" sheetId="1" r:id="rId1"/>
@@ -207,12 +207,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -519,18 +523,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H36"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="27.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="53.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="27.5" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>29</v>
       </c>
@@ -549,12 +553,12 @@
       <c r="F1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>34</v>
       </c>
       <c r="H1"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -573,12 +577,12 @@
       <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="4">
         <v>299607.30011378002</v>
       </c>
       <c r="H2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -597,12 +601,12 @@
       <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="4">
         <v>3593613.2013053601</v>
       </c>
       <c r="H3"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -621,12 +625,12 @@
       <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="4">
         <v>5424241.0516085699</v>
       </c>
       <c r="H4"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -645,11 +649,11 @@
       <c r="F5" t="s">
         <v>18</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="4">
         <v>465873.07765138499</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -668,11 +672,11 @@
       <c r="F6" t="s">
         <v>17</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="4">
         <v>797751.53459731699</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -691,11 +695,11 @@
       <c r="F7" t="s">
         <v>15</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="4">
         <v>412013.84003877599</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -714,11 +718,11 @@
       <c r="F8" t="s">
         <v>16</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="4">
         <v>609463.12967557705</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -737,11 +741,11 @@
       <c r="F9" t="s">
         <v>19</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="4">
         <v>1307300.76</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -760,11 +764,11 @@
       <c r="F10" t="s">
         <v>18</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="4">
         <v>83009.351967474897</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -783,11 +787,11 @@
       <c r="F11" t="s">
         <v>19</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="4">
         <v>4859182.0720829004</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -806,11 +810,11 @@
       <c r="F12" t="s">
         <v>19</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="4">
         <v>12320000</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -829,11 +833,11 @@
       <c r="F13" t="s">
         <v>19</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="4">
         <v>4084775.1528987698</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -852,11 +856,11 @@
       <c r="F14" t="s">
         <v>15</v>
       </c>
-      <c r="G14">
-        <v>497045.44340216101</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G14" s="4">
+        <v>228173.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -875,11 +879,11 @@
       <c r="F15" t="s">
         <v>16</v>
       </c>
-      <c r="G15">
-        <v>1560537.3987719801</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G15" s="4">
+        <v>1063029</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -898,11 +902,11 @@
       <c r="F16" t="s">
         <v>17</v>
       </c>
-      <c r="G16">
-        <v>3334332.4600047702</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G16" s="4">
+        <v>1175444</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -921,11 +925,11 @@
       <c r="F17" t="s">
         <v>18</v>
       </c>
-      <c r="G17">
-        <v>269595.76510894601</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G17" s="4">
+        <v>123332.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -944,11 +948,11 @@
       <c r="F18" t="s">
         <v>15</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -967,11 +971,11 @@
       <c r="F19" t="s">
         <v>16</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="4">
         <v>1000000</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -990,11 +994,11 @@
       <c r="F20" t="s">
         <v>17</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -1013,11 +1017,11 @@
       <c r="F21" t="s">
         <v>18</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1036,11 +1040,11 @@
       <c r="F22" t="s">
         <v>19</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -1059,11 +1063,11 @@
       <c r="F23" t="s">
         <v>19</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -1082,11 +1086,11 @@
       <c r="F24" t="s">
         <v>15</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="4">
         <v>570674.28623627801</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -1105,11 +1109,11 @@
       <c r="F25" t="s">
         <v>20</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="4">
         <v>23472</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -1128,11 +1132,11 @@
       <c r="F26" t="s">
         <v>16</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="4">
         <v>4558948.42278203</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>35</v>
       </c>
@@ -1151,11 +1155,11 @@
       <c r="F27" t="s">
         <v>18</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="4">
         <v>1213156</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -1174,11 +1178,11 @@
       <c r="F28" t="s">
         <v>19</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -1197,11 +1201,11 @@
       <c r="F29" t="s">
         <v>17</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -1220,11 +1224,11 @@
       <c r="F30" t="s">
         <v>24</v>
       </c>
-      <c r="G30">
-        <v>262649.19659017801</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G30" s="4">
+        <v>245448.6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1243,11 +1247,11 @@
       <c r="F31" t="s">
         <v>22</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="4">
         <v>395666.69261358201</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -1266,11 +1270,11 @@
       <c r="F32" t="s">
         <v>26</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="4">
         <v>1820552.416185</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>35</v>
       </c>
@@ -1289,11 +1293,11 @@
       <c r="F33" t="s">
         <v>21</v>
       </c>
-      <c r="G33">
-        <v>469016.42248246103</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G33" s="4">
+        <v>438301.1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1312,11 +1316,11 @@
       <c r="F34" t="s">
         <v>25</v>
       </c>
-      <c r="G34">
-        <v>6106593.8207216403</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G34" s="4">
+        <v>5706680</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -1335,11 +1339,11 @@
       <c r="F35" t="s">
         <v>23</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="4">
         <v>2071325</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -1358,7 +1362,7 @@
       <c r="F36" t="s">
         <v>27</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="4">
         <v>1294172.6187036999</v>
       </c>
     </row>
@@ -1366,4 +1370,10 @@
   <autoFilter ref="A1:G4" xr:uid="{74B3986E-2BCE-704E-B480-617FD308BB93}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>